<commit_message>
Changed in the diff files
</commit_message>
<xml_diff>
--- a/src/test/resources/student_registration.xlsx
+++ b/src/test/resources/student_registration.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Automation\com.ihsm.university.project\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{456EA188-71CB-4377-8172-F914D9F6E6C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92254A5D-AABD-457A-A1C6-1E0E1B8C61B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="961" firstSheet="25" activeTab="26" xr2:uid="{83E1AD02-E6B5-41C8-98D7-77709091ACEC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="961" firstSheet="16" activeTab="18" xr2:uid="{83E1AD02-E6B5-41C8-98D7-77709091ACEC}"/>
   </bookViews>
   <sheets>
     <sheet name="StStatus" sheetId="34" r:id="rId1"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="227">
   <si>
     <t>India</t>
   </si>
@@ -118,9 +118,6 @@
     <t>ID12345</t>
   </si>
   <si>
-    <t>Home Country</t>
-  </si>
-  <si>
     <t>OVNP1234</t>
   </si>
   <si>
@@ -166,9 +163,6 @@
     <t xml:space="preserve"> Haryana (HR) </t>
   </si>
   <si>
-    <t>14 Month Single</t>
-  </si>
-  <si>
     <t>CENTRAL / Bachelor / MBBS</t>
   </si>
   <si>
@@ -746,6 +740,15 @@
   </si>
   <si>
     <t>Latin language (Main)</t>
+  </si>
+  <si>
+    <t>visaAddress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	Russian language (Main)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 11 Months multi </t>
   </si>
 </sst>
 </file>
@@ -1298,7 +1301,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1361,6 +1364,9 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -1741,30 +1747,29 @@
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="D1" s="4" t="s">
         <v>88</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B2" s="2">
         <v>46023</v>
@@ -1773,7 +1778,7 @@
         <v>4554</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -1786,8 +1791,8 @@
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.5546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16.109375" bestFit="1" customWidth="1"/>
@@ -1796,15 +1801,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B2" s="2">
         <v>46023</v>
@@ -1828,24 +1833,24 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C2" s="2">
         <v>46023</v>
@@ -1873,34 +1878,34 @@
     <col min="7" max="7" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="8.33203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.88671875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="14" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="13.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C1" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="D1" s="7" t="s">
         <v>74</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>76</v>
       </c>
       <c r="E1" s="7"/>
       <c r="F1" s="7"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B2" s="1">
         <v>3</v>
@@ -1924,24 +1929,24 @@
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.88671875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="13.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C1" s="7"/>
     </row>
@@ -1965,20 +1970,20 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C1" s="7"/>
     </row>
@@ -2002,26 +2007,26 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="37.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1" s="11" t="s">
         <v>82</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="C1" s="11" t="s">
-        <v>84</v>
       </c>
       <c r="D1" s="13"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B2" s="1">
         <v>121</v>
@@ -2043,36 +2048,36 @@
   <cols>
     <col min="1" max="1" width="10.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.6640625" style="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.5546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.33203125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="8.33203125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="11.88671875" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="14" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="13.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B1" s="8"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B2" s="9"/>
     </row>
@@ -2086,19 +2091,19 @@
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B1" s="8"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -2112,7 +2117,7 @@
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
@@ -2141,18 +2146,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -2173,41 +2178,41 @@
     <col min="6" max="6" width="21.109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="16.5546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="16.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B1" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="E1" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="D1" s="7" t="s">
+      <c r="F1" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="E1" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="F1" s="7" t="s">
-        <v>95</v>
-      </c>
       <c r="G1" s="7" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
@@ -2215,10 +2220,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>28</v>
       </c>
       <c r="D2" s="2">
         <v>44927</v>
@@ -2230,7 +2235,7 @@
         <v>46023</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>0</v>
@@ -2239,7 +2244,7 @@
         <v>7</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -2252,8 +2257,8 @@
   <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.6640625" bestFit="1" customWidth="1"/>
@@ -2267,51 +2272,51 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="E1" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="F1" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="I1" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="D1" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="F1" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="G1" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="H1" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="I1" s="7" t="s">
+      <c r="J1" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="K1" s="7" t="s">
         <v>58</v>
-      </c>
-      <c r="J1" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="K1" s="7" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C2" s="2">
         <v>25569</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E2" s="1">
         <v>91</v>
@@ -2326,10 +2331,10 @@
         <v>0</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>0</v>
@@ -2368,68 +2373,68 @@
   <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="23.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="4.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.5546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="7.88671875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6.88671875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="7.44140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="11" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.77734375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.6640625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="D1" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="E1" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="F1" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="G1" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="H1" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="I1" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="J1" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="K1" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="L1" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="M1" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="N1" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="O1" s="7" t="s">
         <v>58</v>
-      </c>
-      <c r="M1" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="N1" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="O1" s="7" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
@@ -2437,7 +2442,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C2" s="1">
         <v>1</v>
@@ -2449,13 +2454,13 @@
         <v>5</v>
       </c>
       <c r="F2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H2" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>36</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>6</v>
@@ -2473,7 +2478,7 @@
         <v>9876500000</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="O2" s="1" t="s">
         <v>0</v>
@@ -2501,19 +2506,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B1" s="7" t="s">
-        <v>54</v>
-      </c>
       <c r="C1" s="7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -2527,7 +2532,7 @@
         <v>10</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>0</v>
@@ -2550,21 +2555,21 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>50</v>
-      </c>
       <c r="C1" s="4" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B2" s="1">
         <v>5</v>
@@ -2650,36 +2655,36 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="C1" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>125</v>
-      </c>
       <c r="E1" s="4" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D2" s="1">
         <v>1</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>
@@ -2698,84 +2703,84 @@
     <col min="4" max="4" width="12.5546875" customWidth="1"/>
     <col min="5" max="5" width="15" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="18.6640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="20.77734375" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="11.33203125" bestFit="1" customWidth="1"/>
     <col min="16" max="17" width="18" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="16.5546875" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="13.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="E1" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="E1" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="F1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="K1" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="L1" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="M1" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="K1" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="L1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="O1" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="P1" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="Q1" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="R1" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="S1" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="R1" s="4" t="s">
+      <c r="T1" s="4" t="s">
         <v>141</v>
-      </c>
-      <c r="S1" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="T1" s="4" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
@@ -2787,7 +2792,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="F2" s="1">
         <v>900</v>
@@ -2820,7 +2825,7 @@
         <v>40</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="Q2" s="1">
         <v>100</v>
@@ -2849,134 +2854,134 @@
     <col min="2" max="2" width="5.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.44140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="63.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B2" s="1">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" s="1">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>148</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C03AEA9A-D823-42B1-9E97-76ABAEDD901C}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="57" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>128</v>
-      </c>
       <c r="D1" s="4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D2" s="1">
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>225</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>150</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C03AEA9A-D823-42B1-9E97-76ABAEDD901C}">
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="57" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="B2" s="1">
-        <v>1</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="D2" s="1">
-        <v>1</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>225</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="H2" s="6" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -2998,30 +3003,30 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>128</v>
-      </c>
       <c r="D1" s="4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B2" s="9">
         <v>1</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D2" s="9">
         <v>1</v>
@@ -3053,28 +3058,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="C1" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="D1" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="E1" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="F1" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="G1" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="H1" s="7" t="s">
         <v>96</v>
-      </c>
-      <c r="G1" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="H1" s="7" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
@@ -3082,7 +3087,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C2" s="2">
         <v>45658</v>
@@ -3097,7 +3102,7 @@
         <v>85</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H2" s="1">
         <v>90</v>
@@ -3131,10 +3136,10 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>6</v>
@@ -3143,10 +3148,10 @@
         <v>9813981398</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="F2" s="24" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -3163,7 +3168,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="6.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="6" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="4" bestFit="1" customWidth="1"/>
@@ -3194,13 +3199,13 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>36</v>
       </c>
       <c r="D2" s="1">
         <v>25678</v>
@@ -3215,7 +3220,7 @@
         <v>6</v>
       </c>
       <c r="H2" s="24" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="I2" s="2">
         <v>46023</v>
@@ -3227,10 +3232,10 @@
         <v>9813981398</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
   </sheetData>
@@ -3243,7 +3248,7 @@
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="3.33203125" bestFit="1" customWidth="1"/>
@@ -3257,10 +3262,10 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C2" s="2">
         <v>25569</v>
@@ -3279,7 +3284,7 @@
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="3.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3289,10 +3294,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="23" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -3321,7 +3326,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B2" s="1">
         <v>2</v>
@@ -3333,7 +3338,7 @@
         <v>46023</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -3352,7 +3357,7 @@
     <col min="4" max="4" width="6" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.6640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="26.44140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="2" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="10.33203125" bestFit="1" customWidth="1"/>
@@ -3379,13 +3384,13 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B2" s="1">
         <v>0.25</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D2" s="1">
         <v>12589</v>
@@ -3397,13 +3402,13 @@
         <v>46388</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="I2" s="24" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J2" s="1">
         <v>2</v>
@@ -3418,7 +3423,7 @@
         <v>200000</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -3434,7 +3439,7 @@
     <col min="1" max="1" width="16.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3448,7 +3453,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B2" s="2">
         <v>46023</v>
@@ -3457,13 +3462,13 @@
         <v>46388</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -3495,13 +3500,13 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="24" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B2" s="24" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D2" s="1">
         <v>9856</v>
@@ -3513,7 +3518,7 @@
         <v>46388</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -3551,10 +3556,10 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="24" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B2" s="24" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C2" s="2">
         <v>46023</v>
@@ -3563,13 +3568,13 @@
         <v>46388</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="H2" s="1">
         <v>4561</v>
@@ -3578,7 +3583,7 @@
         <v>46753</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -3591,7 +3596,7 @@
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
@@ -3607,10 +3612,10 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C2" s="1">
         <v>523</v>
@@ -3619,7 +3624,7 @@
         <v>46023</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -3634,59 +3639,59 @@
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.88671875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C1" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="D1" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="F1" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="G1" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="H1" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="I1" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="J1" s="7" t="s">
         <v>93</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="F1" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="G1" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="H1" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="I1" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="J1" s="7" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="D2" s="2">
         <v>45292</v>
@@ -3695,13 +3700,13 @@
         <v>45658</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="G2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>26</v>
       </c>
       <c r="I2" s="22">
         <v>88</v>
@@ -3749,28 +3754,28 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="24" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B2" s="2">
         <v>46023</v>
       </c>
       <c r="C2" s="24" t="s">
+        <v>218</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="E2" s="24" t="s">
         <v>220</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="F2" s="24" t="s">
         <v>221</v>
       </c>
-      <c r="E2" s="24" t="s">
+      <c r="G2" s="24" t="s">
         <v>222</v>
       </c>
-      <c r="F2" s="24" t="s">
-        <v>223</v>
-      </c>
-      <c r="G2" s="24" t="s">
-        <v>224</v>
-      </c>
       <c r="H2" s="24" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -3808,13 +3813,13 @@
         <v>46023</v>
       </c>
       <c r="C2" s="24" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="D2" s="1">
         <v>246</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -3827,7 +3832,7 @@
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="32.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
@@ -3848,16 +3853,16 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="B2" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="B2" s="24" t="s">
+      <c r="D2" s="24" t="s">
         <v>208</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="D2" s="24" t="s">
-        <v>210</v>
       </c>
       <c r="E2" s="1">
         <v>589</v>
@@ -3866,10 +3871,10 @@
         <v>46023</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
   </sheetData>
@@ -3882,9 +3887,9 @@
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="3.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="3.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.44140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.109375" bestFit="1" customWidth="1"/>
@@ -3900,22 +3905,22 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>204</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>206</v>
       </c>
       <c r="E2" s="2">
         <v>46023</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -3942,7 +3947,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B2" s="1">
         <v>2598</v>
@@ -3951,7 +3956,7 @@
         <v>46023</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -3977,7 +3982,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -3992,7 +3997,7 @@
   <cols>
     <col min="1" max="1" width="11.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
@@ -4011,22 +4016,22 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>197</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>199</v>
       </c>
       <c r="D2" s="1">
         <v>1256</v>
       </c>
       <c r="E2" s="24" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="F2" s="24" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="G2" s="2">
         <v>46023</v>
@@ -4047,71 +4052,72 @@
   <cols>
     <col min="1" max="1" width="15.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="11.88671875" customWidth="1"/>
-    <col min="10" max="11" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="4.44140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="4.5546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="L1" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="E1" s="4" t="s">
+      <c r="M1" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="L1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="M1" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D2" s="1">
         <v>1</v>
@@ -4120,16 +4126,16 @@
         <v>1</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>171</v>
+        <v>162</v>
+      </c>
+      <c r="H2" s="25" t="s">
+        <v>159</v>
       </c>
       <c r="I2" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J2" s="2">
         <v>46055</v>
@@ -4138,13 +4144,13 @@
         <v>46083</v>
       </c>
       <c r="L2" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="N2" s="1" t="s">
         <v>157</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>159</v>
       </c>
     </row>
   </sheetData>
@@ -4162,68 +4168,68 @@
     <col min="3" max="3" width="23.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.5546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.44140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.88671875" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="10" max="11" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="8.5546875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="34.77734375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="34.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="L1" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="E1" s="4" t="s">
+      <c r="M1" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="L1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>154</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D2" s="1">
         <v>1</v>
@@ -4232,13 +4238,13 @@
         <v>1</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="I2" s="1">
         <v>3</v>
@@ -4250,13 +4256,13 @@
         <v>46083</v>
       </c>
       <c r="L2" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="N2" s="1" t="s">
         <v>172</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -4280,70 +4286,70 @@
     <col min="9" max="10" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="11" max="12" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="22.77734375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="22.6640625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="34.77734375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="34.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="M1" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="E1" s="4" t="s">
+      <c r="N1" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="O1" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="M1" s="4" t="s">
+      <c r="P1" s="4" t="s">
         <v>154</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D2" s="1">
         <v>1</v>
@@ -4352,16 +4358,16 @@
         <v>1</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="J2" s="1">
         <v>2</v>
@@ -4373,16 +4379,16 @@
         <v>46083</v>
       </c>
       <c r="M2" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="P2" s="1" t="s">
         <v>172</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -4395,14 +4401,13 @@
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="15" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
@@ -4429,16 +4434,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -4465,51 +4470,49 @@
   <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="6" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.77734375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I1" s="19" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>16</v>
-      </c>
+        <v>226</v>
+      </c>
+      <c r="B2" s="1"/>
       <c r="C2" s="2">
         <v>47484</v>
       </c>
@@ -4523,13 +4526,13 @@
         <v>49310</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="I2" s="16" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -4539,48 +4542,53 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{183CB891-07B1-419C-9500-43DAB1CEB717}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>93</v>
+        <v>224</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>111</v>
+        <v>92</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+        <v>109</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B2" s="2">
+        <v>226</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="2">
         <v>49310</v>
       </c>
-      <c r="C2" s="2">
+      <c r="D2" s="2">
         <v>50406</v>
       </c>
-      <c r="D2" s="2">
+      <c r="E2" s="2">
         <v>51136</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>17</v>
+      <c r="F2" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -4601,22 +4609,20 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>16</v>
-      </c>
+      <c r="A2" s="1"/>
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -4624,7 +4630,7 @@
         <v>46023</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -4633,21 +4639,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C8BB2145AC5254468C792DE10D43AC94" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2e5a2447409261ea00061a7e0347d58b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="facf0261-3046-4379-83e6-4b564f239035" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="60aaf839d7127e9db1ed69495fc40e99" ns3:_="">
     <xsd:import namespace="facf0261-3046-4379-83e6-4b564f239035"/>
@@ -4791,31 +4782,22 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51273304-BDAD-4DD0-B8B1-1249F784DB7A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="facf0261-3046-4379-83e6-4b564f239035"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD24E627-8D77-45E6-A2E8-6D72477AEF2F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A7BBEB4-EFA4-4BBC-AEC4-BF9096A43876}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4831,4 +4813,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51273304-BDAD-4DD0-B8B1-1249F784DB7A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="facf0261-3046-4379-83e6-4b564f239035"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD24E627-8D77-45E6-A2E8-6D72477AEF2F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>